<commit_message>
Implement agent stream (GStreamer -> OpenCV -> ROS2)
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Multi-Target-Heterogeneus.xlsx
+++ b/src/flychams_common/config/Configuration-Multi-Target-Heterogeneus.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="264">
   <si>
     <t xml:space="preserve">GENERAL CONFIGURATION</t>
   </si>
@@ -226,9 +226,6 @@
     <t xml:space="preserve">BatteryCapacity [mAh]</t>
   </si>
   <si>
-    <t xml:space="preserve">InferenceStreamURL</t>
-  </si>
-  <si>
     <t xml:space="preserve">AGENT00</t>
   </si>
   <si>
@@ -247,9 +244,6 @@
     <t xml:space="preserve">(Roll=0.0, Pitch=0.0, Yaw=0.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">tcp://127.0.0.1:5500</t>
-  </si>
-  <si>
     <t xml:space="preserve">AGENT01</t>
   </si>
   <si>
@@ -262,9 +256,6 @@
     <t xml:space="preserve">(X=-10.0, Y=0.0, Z=0.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">tcp://127.0.0.1:5501</t>
-  </si>
-  <si>
     <t xml:space="preserve">AGENT02</t>
   </si>
   <si>
@@ -277,9 +268,6 @@
     <t xml:space="preserve">(X=0.0, Y=10.0, Z=0.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">tcp://127.0.0.1:5502</t>
-  </si>
-  <si>
     <t xml:space="preserve">AGENT03</t>
   </si>
   <si>
@@ -406,9 +394,6 @@
     <t xml:space="preserve">SourceStreamURL</t>
   </si>
   <si>
-    <t xml:space="preserve">InterfaceStreamURL</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hardware</t>
   </si>
   <si>
@@ -439,10 +424,7 @@
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=90.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">udp://127.0.0.1:5000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">udp://127.0.0.1:6000</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT00/MULTICAMERA00</t>
   </si>
   <si>
     <t xml:space="preserve">SIYI A8 Mini</t>
@@ -469,10 +451,7 @@
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=0.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">udp://127.0.0.1:5001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">udp://127.0.0.1:6001</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT00/MULTICAMERA01</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA02</t>
@@ -484,10 +463,7 @@
     <t xml:space="preserve">(X=0.0, Y=0.3, Z=-0.05)</t>
   </si>
   <si>
-    <t xml:space="preserve">udp://127.0.0.1:5002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">udp://127.0.0.1:6002</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT00/MULTICAMERA02</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA03</t>
@@ -496,10 +472,7 @@
     <t xml:space="preserve">Central Head 2 Multi-Camera (2 Cameras)</t>
   </si>
   <si>
-    <t xml:space="preserve">udp://127.0.0.1:5003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">udp://127.0.0.1:6003</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT01/MULTICAMERA03</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA04</t>
@@ -508,10 +481,7 @@
     <t xml:space="preserve">Tracking Head 2.1 Multi-Camera (2 Cameras)</t>
   </si>
   <si>
-    <t xml:space="preserve">udp://127.0.0.1:5004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">udp://127.0.0.1:6004</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT01/MULTICAMERA04</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA05</t>
@@ -520,10 +490,7 @@
     <t xml:space="preserve">Tracking Head 2.2 Multi-Camera (2 Cameras)</t>
   </si>
   <si>
-    <t xml:space="preserve">udp://127.0.0.1:5005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">udp://127.0.0.1:6005</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT01/MULTICAMERA05</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA06</t>
@@ -532,10 +499,7 @@
     <t xml:space="preserve">Central Head 3 Multi-Camera (2 Cameras)</t>
   </si>
   <si>
-    <t xml:space="preserve">udp://127.0.0.1:5006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">udp://127.0.0.1:6006</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT02/MULTICAMERA06</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA07</t>
@@ -544,10 +508,7 @@
     <t xml:space="preserve">Tracking Head 3.1 Multi-Camera (2 Cameras)</t>
   </si>
   <si>
-    <t xml:space="preserve">udp://127.0.0.1:5007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">udp://127.0.0.1:6007</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT02/MULTICAMERA07</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA08</t>
@@ -556,10 +517,7 @@
     <t xml:space="preserve">Tracking Head 3.2 Multi-Camera (2 Cameras)</t>
   </si>
   <si>
-    <t xml:space="preserve">udp://127.0.0.1:5008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">udp://127.0.0.1:6008</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT02/MULTICAMERA08</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA09</t>
@@ -571,13 +529,16 @@
     <t xml:space="preserve">CAM02</t>
   </si>
   <si>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT03/MULTICAMERA09</t>
+  </si>
+  <si>
     <t xml:space="preserve">MULTICAMERA10</t>
   </si>
   <si>
     <t xml:space="preserve">Central Head 2 Multi-Window (2 Windows)</t>
   </si>
   <si>
-    <t xml:space="preserve">Udp://127.0.0.1:6003</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT04/MULTICAMERA10</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA11</t>
@@ -586,7 +547,7 @@
     <t xml:space="preserve">Central Head 3 Multi-Window (2 Windows)</t>
   </si>
   <si>
-    <t xml:space="preserve">Udp://127.0.0.1:6006</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT05/MULTICAMERA11</t>
   </si>
   <si>
     <t xml:space="preserve">MULTICAMERA12</t>
@@ -595,18 +556,27 @@
     <t xml:space="preserve">Central Head 1 Multi-Camera (3 Cameras)</t>
   </si>
   <si>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT06/MULTICAMERA12</t>
+  </si>
+  <si>
     <t xml:space="preserve">MULTICAMERA13</t>
   </si>
   <si>
     <t xml:space="preserve">Tracking Head 1.1 Multi-Camera (3 Cameras)</t>
   </si>
   <si>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT06/MULTICAMERA13</t>
+  </si>
+  <si>
     <t xml:space="preserve">MULTICAMERA14</t>
   </si>
   <si>
     <t xml:space="preserve">Tracking Head 1.2 Multi-Camera (3 Cameras)</t>
   </si>
   <si>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT06/MULTICAMERA14</t>
+  </si>
+  <si>
     <t xml:space="preserve">MULTICAMERA15</t>
   </si>
   <si>
@@ -619,10 +589,16 @@
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=180.0)</t>
   </si>
   <si>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT06/MULTICAMERA15</t>
+  </si>
+  <si>
     <t xml:space="preserve">MULTICAMERA16</t>
   </si>
   <si>
     <t xml:space="preserve">Central Head 2 Multi-Window (3 Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT07/MULTICAMERA16</t>
   </si>
   <si>
     <t xml:space="preserve">Resolution [pix]</t>
@@ -1242,9 +1218,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:K2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A2:K2"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:J2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A2:J2"/>
+  <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Name"/>
     <tableColumn id="3" name="AgentTeamID"/>
@@ -1255,7 +1231,6 @@
     <tableColumn id="8" name="MaxAltitude [m]"/>
     <tableColumn id="9" name="SafetyRadius [m]"/>
     <tableColumn id="10" name="BatteryCapacity [mAh]"/>
-    <tableColumn id="11" name="InferenceStreamURL"/>
   </tableColumns>
 </table>
 </file>
@@ -1934,7 +1909,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1955,62 +1930,62 @@
         <v>2</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="C3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="E3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="I3" s="21" t="n">
         <v>0.4</v>
@@ -2601,7 +2576,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:XFD1048576"/>
+  <dimension ref="A1:XFD13"/>
   <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
@@ -2612,11 +2587,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="29.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="36.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="2" width="26.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="2" width="29.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="26.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="17" min="13" style="12" width="11"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16380" min="18" style="2" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="3" width="10.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="29.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="11.44"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16" min="12" style="12" width="11"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16379" min="17" style="2" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16380" min="16380" style="0" width="10.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16383" min="16381" style="3" width="10.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="3" width="10.58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2632,7 +2609,6 @@
       <c r="H1" s="16"/>
       <c r="I1" s="16"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
@@ -2665,14 +2641,12 @@
       <c r="J2" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="K2" s="17" t="s">
-        <v>65</v>
-      </c>
+      <c r="L2" s="12"/>
       <c r="M2" s="12"/>
       <c r="N2" s="12"/>
       <c r="O2" s="12"/>
       <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
+      <c r="XEZ2" s="0"/>
       <c r="XFA2" s="3"/>
       <c r="XFB2" s="3"/>
       <c r="XFC2" s="3"/>
@@ -2680,25 +2654,25 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="18" t="s">
         <v>66</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>67</v>
       </c>
       <c r="C3" s="18" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="F3" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="G3" s="18" t="s">
         <v>70</v>
-      </c>
-      <c r="G3" s="18" t="s">
-        <v>71</v>
       </c>
       <c r="H3" s="18" t="n">
         <v>300</v>
@@ -2709,31 +2683,28 @@
       <c r="J3" s="18" t="n">
         <v>12000</v>
       </c>
-      <c r="K3" s="18" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H4" s="18" t="n">
         <v>300</v>
@@ -2744,31 +2715,28 @@
       <c r="J4" s="18" t="n">
         <v>12000</v>
       </c>
-      <c r="K4" s="18" t="s">
-        <v>77</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C5" s="18" t="s">
         <v>16</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H5" s="18" t="n">
         <v>300</v>
@@ -2779,31 +2747,28 @@
       <c r="J5" s="18" t="n">
         <v>12000</v>
       </c>
-      <c r="K5" s="18" t="s">
-        <v>82</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C6" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E6" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="F6" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="G6" s="18" t="s">
         <v>70</v>
-      </c>
-      <c r="G6" s="18" t="s">
-        <v>71</v>
       </c>
       <c r="H6" s="18" t="n">
         <v>300</v>
@@ -2814,31 +2779,28 @@
       <c r="J6" s="18" t="n">
         <v>12000</v>
       </c>
-      <c r="K6" s="18" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C7" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H7" s="18" t="n">
         <v>300</v>
@@ -2849,31 +2811,28 @@
       <c r="J7" s="18" t="n">
         <v>12000</v>
       </c>
-      <c r="K7" s="18" t="s">
-        <v>77</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C8" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H8" s="18" t="n">
         <v>300</v>
@@ -2884,31 +2843,28 @@
       <c r="J8" s="18" t="n">
         <v>12000</v>
       </c>
-      <c r="K8" s="18" t="s">
-        <v>82</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E9" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="G9" s="18" t="s">
         <v>70</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>71</v>
       </c>
       <c r="H9" s="18" t="n">
         <v>300</v>
@@ -2919,31 +2875,28 @@
       <c r="J9" s="18" t="n">
         <v>12000</v>
       </c>
-      <c r="K9" s="18" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C10" s="18" t="s">
         <v>27</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H10" s="18" t="n">
         <v>300</v>
@@ -2953,18 +2906,14 @@
       </c>
       <c r="J10" s="18" t="n">
         <v>12000</v>
-      </c>
-      <c r="K10" s="18" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="12" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3018,16 +2967,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="H2" s="12"/>
       <c r="I2" s="12"/>
@@ -3043,13 +2992,13 @@
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D3" s="18" t="n">
         <v>0.2</v>
@@ -3068,13 +3017,13 @@
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D4" s="18" t="n">
         <v>0.2</v>
@@ -3098,13 +3047,13 @@
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D5" s="18" t="n">
         <v>0.2</v>
@@ -3128,13 +3077,13 @@
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D6" s="18" t="n">
         <v>0.2</v>
@@ -3153,13 +3102,13 @@
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>0.2</v>
@@ -3178,13 +3127,13 @@
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>0.2</v>
@@ -3203,13 +3152,13 @@
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D9" s="18" t="n">
         <v>0.2</v>
@@ -3228,13 +3177,13 @@
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D10" s="18" t="n">
         <v>0.2</v>
@@ -3289,7 +3238,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:T1048576"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.34"/>
@@ -3298,13 +3247,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="12" width="27.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="36.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="2" width="27.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="37.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="30.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="27.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="2" width="21.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="2" width="16.23"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="20" min="17" style="12" width="11"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="21" style="2" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="54.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="27.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="21.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="2" width="16.23"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="19" min="16" style="12" width="11"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16383" min="21" style="2" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="2" width="10.58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3325,7 +3274,6 @@
       <c r="M1" s="16"/>
       <c r="N1" s="16"/>
       <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
@@ -3335,16 +3283,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="G2" s="17" t="s">
         <v>60</v>
@@ -3353,58 +3301,56 @@
         <v>61</v>
       </c>
       <c r="I2" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="J2" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="L2" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="M2" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="N2" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="O2" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="L2" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="M2" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="N2" s="17" t="s">
-        <v>126</v>
-      </c>
-      <c r="O2" s="17" t="s">
-        <v>127</v>
-      </c>
-      <c r="P2" s="17" t="s">
-        <v>128</v>
-      </c>
+      <c r="P2" s="12"/>
       <c r="Q2" s="12"/>
       <c r="R2" s="12"/>
       <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
+      <c r="T2" s="0"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="G3" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="H3" s="18" t="s">
         <v>130</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>103</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="E3" s="18" t="s">
-        <v>132</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="G3" s="18" t="s">
-        <v>134</v>
-      </c>
-      <c r="H3" s="18" t="s">
-        <v>135</v>
       </c>
       <c r="I3" s="18" t="n">
         <v>3</v>
@@ -3416,45 +3362,43 @@
         <v>3</v>
       </c>
       <c r="L3" s="18" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O3" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P3" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O3" s="18" t="n">
         <v>37260</v>
       </c>
+      <c r="T3" s="0"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="I4" s="18" t="n">
         <v>8</v>
@@ -3466,45 +3410,43 @@
         <v>10</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O4" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P4" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O4" s="18" t="n">
         <v>37260</v>
       </c>
+      <c r="T4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F5" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="G5" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="G5" s="18" t="s">
-        <v>150</v>
-      </c>
       <c r="H5" s="18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I5" s="18" t="n">
         <v>8</v>
@@ -3516,45 +3458,42 @@
         <v>10</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="M5" s="18" t="s">
-        <v>152</v>
+        <v>132</v>
       </c>
       <c r="N5" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O5" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P5" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O5" s="18" t="n">
         <v>37260</v>
       </c>
     </row>
     <row r="6" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I6" s="18" t="n">
         <v>3</v>
@@ -3566,49 +3505,47 @@
         <v>3</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>156</v>
+        <v>132</v>
       </c>
       <c r="N6" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O6" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P6" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O6" s="18" t="n">
         <v>37260</v>
       </c>
+      <c r="P6" s="12"/>
       <c r="Q6" s="12"/>
       <c r="R6" s="12"/>
       <c r="S6" s="12"/>
-      <c r="T6" s="12"/>
+      <c r="T6" s="0"/>
     </row>
     <row r="7" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="I7" s="18" t="n">
         <v>8</v>
@@ -3620,49 +3557,47 @@
         <v>10</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>160</v>
+        <v>132</v>
       </c>
       <c r="N7" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O7" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P7" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O7" s="18" t="n">
         <v>37260</v>
       </c>
+      <c r="P7" s="12"/>
       <c r="Q7" s="12"/>
       <c r="R7" s="12"/>
       <c r="S7" s="12"/>
-      <c r="T7" s="12"/>
+      <c r="T7" s="0"/>
     </row>
     <row r="8" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F8" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="G8" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="G8" s="18" t="s">
-        <v>150</v>
-      </c>
       <c r="H8" s="18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I8" s="18" t="n">
         <v>8</v>
@@ -3674,49 +3609,47 @@
         <v>10</v>
       </c>
       <c r="L8" s="18" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="M8" s="18" t="s">
-        <v>164</v>
+        <v>132</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O8" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P8" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O8" s="18" t="n">
         <v>37260</v>
       </c>
+      <c r="P8" s="12"/>
       <c r="Q8" s="12"/>
       <c r="R8" s="12"/>
       <c r="S8" s="12"/>
-      <c r="T8" s="12"/>
+      <c r="T8" s="0"/>
     </row>
     <row r="9" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I9" s="18" t="n">
         <v>3</v>
@@ -3728,49 +3661,47 @@
         <v>3</v>
       </c>
       <c r="L9" s="18" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="M9" s="18" t="s">
-        <v>168</v>
+        <v>132</v>
       </c>
       <c r="N9" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O9" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P9" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O9" s="18" t="n">
         <v>37260</v>
       </c>
+      <c r="P9" s="12"/>
       <c r="Q9" s="12"/>
       <c r="R9" s="12"/>
       <c r="S9" s="12"/>
-      <c r="T9" s="12"/>
+      <c r="T9" s="0"/>
     </row>
     <row r="10" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="I10" s="18" t="n">
         <v>8</v>
@@ -3782,49 +3713,47 @@
         <v>10</v>
       </c>
       <c r="L10" s="18" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="M10" s="18" t="s">
-        <v>172</v>
+        <v>132</v>
       </c>
       <c r="N10" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O10" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P10" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O10" s="18" t="n">
         <v>37260</v>
       </c>
+      <c r="P10" s="12"/>
       <c r="Q10" s="12"/>
       <c r="R10" s="12"/>
       <c r="S10" s="12"/>
-      <c r="T10" s="12"/>
+      <c r="T10" s="0"/>
     </row>
     <row r="11" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F11" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="G11" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="G11" s="18" t="s">
-        <v>150</v>
-      </c>
       <c r="H11" s="18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I11" s="18" t="n">
         <v>8</v>
@@ -3836,49 +3765,47 @@
         <v>10</v>
       </c>
       <c r="L11" s="18" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="M11" s="18" t="s">
-        <v>176</v>
+        <v>132</v>
       </c>
       <c r="N11" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O11" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P11" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O11" s="18" t="n">
         <v>37260</v>
       </c>
+      <c r="P11" s="12"/>
       <c r="Q11" s="12"/>
       <c r="R11" s="12"/>
       <c r="S11" s="12"/>
-      <c r="T11" s="12"/>
+      <c r="T11" s="0"/>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>178</v>
+        <v>164</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I12" s="18" t="n">
         <v>3</v>
@@ -3890,45 +3817,42 @@
         <v>3</v>
       </c>
       <c r="L12" s="18" t="s">
-        <v>136</v>
+        <v>166</v>
       </c>
       <c r="M12" s="18" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="N12" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O12" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P12" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O12" s="18" t="n">
         <v>37260</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I13" s="18" t="n">
         <v>3</v>
@@ -3940,45 +3864,42 @@
         <v>3</v>
       </c>
       <c r="L13" s="18" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="M13" s="18" t="s">
-        <v>182</v>
+        <v>132</v>
       </c>
       <c r="N13" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O13" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P13" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O13" s="18" t="n">
         <v>37260</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>183</v>
+        <v>170</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>184</v>
+        <v>171</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I14" s="18" t="n">
         <v>3</v>
@@ -3990,45 +3911,42 @@
         <v>3</v>
       </c>
       <c r="L14" s="18" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="M14" s="18" t="s">
-        <v>185</v>
+        <v>132</v>
       </c>
       <c r="N14" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O14" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P14" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O14" s="18" t="n">
         <v>37260</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I15" s="18" t="n">
         <v>3</v>
@@ -4040,45 +3958,42 @@
         <v>3</v>
       </c>
       <c r="L15" s="18" t="s">
-        <v>136</v>
+        <v>175</v>
       </c>
       <c r="M15" s="18" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="N15" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O15" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P15" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O15" s="18" t="n">
         <v>37260</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="H16" s="18" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="I16" s="18" t="n">
         <v>8</v>
@@ -4090,45 +4005,42 @@
         <v>10</v>
       </c>
       <c r="L16" s="18" t="s">
-        <v>146</v>
+        <v>178</v>
       </c>
       <c r="M16" s="18" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="N16" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O16" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P16" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O16" s="18" t="n">
         <v>37260</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F17" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="G17" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="G17" s="18" t="s">
-        <v>150</v>
-      </c>
       <c r="H17" s="18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I17" s="18" t="n">
         <v>8</v>
@@ -4140,45 +4052,42 @@
         <v>10</v>
       </c>
       <c r="L17" s="18" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
       <c r="M17" s="18" t="s">
-        <v>152</v>
+        <v>132</v>
       </c>
       <c r="N17" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O17" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P17" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O17" s="18" t="n">
         <v>37260</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="I18" s="18" t="n">
         <v>8</v>
@@ -4190,45 +4099,42 @@
         <v>10</v>
       </c>
       <c r="L18" s="18" t="s">
-        <v>155</v>
+        <v>186</v>
       </c>
       <c r="M18" s="18" t="s">
-        <v>156</v>
+        <v>132</v>
       </c>
       <c r="N18" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O18" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P18" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O18" s="18" t="n">
         <v>37260</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="G19" s="18" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="H19" s="18" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I19" s="18" t="n">
         <v>3</v>
@@ -4240,43 +4146,21 @@
         <v>3</v>
       </c>
       <c r="L19" s="18" t="s">
-        <v>159</v>
+        <v>189</v>
       </c>
       <c r="M19" s="18" t="s">
-        <v>160</v>
+        <v>132</v>
       </c>
       <c r="N19" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="O19" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P19" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="O19" s="18" t="n">
         <v>37260</v>
       </c>
     </row>
-    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4296,7 +4180,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:XFD1048576"/>
+  <dimension ref="A1:XFD17"/>
   <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.34"/>
@@ -4305,9 +4189,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="12" width="27.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="2" width="27.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="12" width="27.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="32.56"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16375" min="9" style="2" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16376" style="3" width="10.49"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16374" min="8" style="2" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16375" min="16375" style="0" width="10.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16383" min="16376" style="3" width="10.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="3" width="10.58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4320,7 +4205,6 @@
       <c r="E1" s="16"/>
       <c r="F1" s="16"/>
       <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
@@ -4330,23 +4214,21 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>201</v>
-      </c>
-      <c r="H2" s="17" t="s">
-        <v>125</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="XEU2" s="0"/>
       <c r="XEV2" s="3"/>
       <c r="XEW2" s="3"/>
       <c r="XEX2" s="3"/>
@@ -4359,16 +4241,16 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="E3" s="18" t="n">
         <v>0.167</v>
@@ -4379,22 +4261,19 @@
       <c r="G3" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="H3" s="18" t="s">
-        <v>147</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="E4" s="18" t="n">
         <v>0.167</v>
@@ -4405,22 +4284,19 @@
       <c r="G4" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="H4" s="18" t="s">
-        <v>152</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="E5" s="18" t="n">
         <v>0.167</v>
@@ -4431,22 +4307,19 @@
       <c r="G5" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="H5" s="18" t="s">
-        <v>160</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="E6" s="18" t="n">
         <v>0.167</v>
@@ -4457,22 +4330,19 @@
       <c r="G6" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="H6" s="18" t="s">
-        <v>164</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="E7" s="18" t="n">
         <v>0.167</v>
@@ -4483,22 +4353,19 @@
       <c r="G7" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="H7" s="18" t="s">
-        <v>172</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="E8" s="18" t="n">
         <v>0.167</v>
@@ -4509,22 +4376,19 @@
       <c r="G8" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="H8" s="18" t="s">
-        <v>176</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="E9" s="18" t="n">
         <v>0.167</v>
@@ -4535,22 +4399,19 @@
       <c r="G9" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="H9" s="18" t="s">
-        <v>164</v>
-      </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="E10" s="18" t="n">
         <v>0.167</v>
@@ -4561,22 +4422,19 @@
       <c r="G10" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="H10" s="18" t="s">
-        <v>168</v>
-      </c>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="E11" s="18" t="n">
         <v>0.167</v>
@@ -4587,51 +4445,16 @@
       <c r="G11" s="18" t="n">
         <v>0.583</v>
       </c>
-      <c r="H11" s="18" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H12" s="12"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H13" s="12"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H14" s="12"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H15" s="12"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H16" s="12"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H17" s="12"/>
-    </row>
-    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4671,7 +4494,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -4702,60 +4525,60 @@
         <v>36</v>
       </c>
       <c r="D2" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="G2" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="H2" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="I2" s="20" t="s">
+        <v>219</v>
+      </c>
+      <c r="J2" s="20" t="s">
+        <v>220</v>
+      </c>
+      <c r="K2" s="20" t="s">
+        <v>221</v>
+      </c>
+      <c r="L2" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="M2" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="N2" s="20" t="s">
         <v>224</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="O2" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="H2" s="20" t="s">
+      <c r="P2" s="20" t="s">
         <v>226</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="Q2" s="20" t="s">
         <v>227</v>
       </c>
-      <c r="J2" s="20" t="s">
+      <c r="R2" s="20" t="s">
         <v>228</v>
-      </c>
-      <c r="K2" s="20" t="s">
-        <v>229</v>
-      </c>
-      <c r="L2" s="20" t="s">
-        <v>230</v>
-      </c>
-      <c r="M2" s="20" t="s">
-        <v>231</v>
-      </c>
-      <c r="N2" s="20" t="s">
-        <v>232</v>
-      </c>
-      <c r="O2" s="20" t="s">
-        <v>233</v>
-      </c>
-      <c r="P2" s="20" t="s">
-        <v>234</v>
-      </c>
-      <c r="Q2" s="20" t="s">
-        <v>235</v>
-      </c>
-      <c r="R2" s="20" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="D3" s="21" t="n">
         <v>8</v>
@@ -4768,28 +4591,28 @@
         <v>1</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="H3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I3" s="21" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="J3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K3" s="21" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="L3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="N3" s="21" t="n">
         <v>6.5</v>
@@ -4864,7 +4687,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -4888,28 +4711,28 @@
         <v>36</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="XFB2" s="3"/>
       <c r="XFC2" s="3"/>
@@ -4917,29 +4740,29 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="I3" s="21" t="n">
         <v>0.5</v>
@@ -4953,29 +4776,29 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="G4" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="I4" s="21" t="n">
         <v>0.5</v>
@@ -4989,29 +4812,29 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="C5" s="21" t="s">
+        <v>243</v>
+      </c>
+      <c r="D5" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="D5" s="21" t="s">
-        <v>259</v>
-      </c>
       <c r="E5" s="21" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="G5" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="I5" s="21" t="n">
         <v>0.5</v>

</xml_diff>